<commit_message>
Finished unittesting InvestmentAccount everything works as intended
</commit_message>
<xml_diff>
--- a/tests/A02_pixell_test_plan_chequing_account.xlsx
+++ b/tests/A02_pixell_test_plan_chequing_account.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1c7409c97bef83d8/Desktop/School/Term 2/ISD/Assignments/Donald_Trevor_Assignment/tests/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36C6C282-9E95-49F5-8B02-013BC46A4462}"/>
+  <xr:revisionPtr revIDLastSave="37" documentId="13_ncr:1_{2873F10E-F8B1-4F89-8CDF-A98B96DD770E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75355610-77CF-40F7-B505-3853ABB4C08E}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-21600" windowWidth="26010" windowHeight="20985" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
+    <workbookView xWindow="-14640" yWindow="-2850" windowWidth="12150" windowHeight="20745" xr2:uid="{8D9DD509-55B1-455D-8036-16809AD15960}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -183,7 +183,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="40">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -300,6 +300,9 @@
   </si>
   <si>
     <t xml:space="preserve">Account Number: 123 Balance: $1,050.50                          Overdraft Limit: $-50 Overdraft Rate: 2% Account Type: Chequing   </t>
+  </si>
+  <si>
+    <t>Trevor Donald</t>
   </si>
 </sst>
 </file>
@@ -806,6 +809,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1231,7 +1238,9 @@
       <c r="B3" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="16"/>
+      <c r="C3" s="16" t="s">
+        <v>39</v>
+      </c>
       <c r="D3" s="17"/>
     </row>
     <row r="4" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>